<commit_message>
docs: record the removed and changed variables in the workbook
The documentation sheet still described UseSubplots and xSliderStep as if
they worked, and said nothing about blocks or the X range boxes. Appended a
dated section covering all four, so the reference beside the settings agrees
with the code.

Edited through the workbook's own XML, one zip entry at a time, so the
printerSettings parts survive; openpyxl drops them. dash-config.json is
regenerated from it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dash-config.xlsx
+++ b/dash-config.xlsx
@@ -3327,7 +3327,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:AMK75"/>
+  <dimension ref="A1:AMK86"/>
   <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.69140625" style="12" customWidth="1"/>
@@ -10997,6 +10997,89 @@
         </is>
       </c>
     </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Changed 2026-09-11:</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Also opens a BLOCK: rows below it apply to the graphs below it</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>A second Height starts a new block, which may name its own Datafile</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>A block inherits xValue and xLabel from above if it does not set them</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>This is how one tab carries several data files at different rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>UseSubplots</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>REMOVED. Had been disabled for some time. Use blocks and commonX instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>xSliderStep</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>REMOVED with the x-axis slider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>X range boxes</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Beside each graph: type a start and an end, Apply to zoom, Reset to undo</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Replaces the old slider. On a commonX tab it drives every graph on the tab.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A9:B9"/>

</xml_diff>